<commit_message>
se añade test de correo duplicado
</commit_message>
<xml_diff>
--- a/Registro_Pruebas_Unitarias.xlsx
+++ b/Registro_Pruebas_Unitarias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moka/Documents/ReactPasteleria/ProyectoReactPasteleria/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F234EF2-274D-9E47-A3A7-73F9E7CA35A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738BECD4-3BAC-DA4F-9364-80FB319E7D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="20000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,187 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="93">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Módulo / Clase</t>
+  </si>
+  <si>
+    <t>Función / Método</t>
+  </si>
+  <si>
+    <t>Tipo de caso</t>
+  </si>
+  <si>
+    <t>Descripción del caso</t>
+  </si>
+  <si>
+    <t>Datos de entrada</t>
+  </si>
+  <si>
+    <t>Resultado esperado</t>
+  </si>
+  <si>
+    <t>Resultado obtenido</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Responsable</t>
+  </si>
+  <si>
+    <t>Fecha ejecución</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>PU-001</t>
+  </si>
+  <si>
+    <t>Carrito</t>
+  </si>
+  <si>
+    <t>agregarAlCarrito(codigo)</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Agregar dos veces el mismo producto (TC001) deja una sola fila con cantidad 2</t>
+  </si>
+  <si>
+    <t>codigo: 'TC001' (dos clicks en 'Agregar Torta')</t>
+  </si>
+  <si>
+    <t>Una sola fila TC001 con cantidad 2 y totalUnidades = 2</t>
+  </si>
+  <si>
+    <t>Se muestra 'Items: TC001x2' y 'Unidades: 2'</t>
+  </si>
+  <si>
+    <t>Pasó</t>
+  </si>
+  <si>
+    <t>Joaquin Fuenzalida</t>
+  </si>
+  <si>
+    <t>PU-002</t>
+  </si>
+  <si>
+    <t>agregarAlCarrito - persistencia (localStorage)</t>
+  </si>
+  <si>
+    <t>El carrito se guarda en localStorage al agregar un producto</t>
+  </si>
+  <si>
+    <t>codigo: 'TC001'</t>
+  </si>
+  <si>
+    <t>localStorage['carrito'] contiene 1 item TC001 con cantidad 1</t>
+  </si>
+  <si>
+    <t>carrito = [{ codigo: 'TC001', cantidad: 1 }]</t>
+  </si>
+  <si>
+    <t>PU-003</t>
+  </si>
+  <si>
+    <t>vaciarCarrito()</t>
+  </si>
+  <si>
+    <t>Borde</t>
+  </si>
+  <si>
+    <t>Vaciar el carrito deja el carrito y localStorage vacíos</t>
+  </si>
+  <si>
+    <t>Agregar TC001 y luego click en 'Vaciar'</t>
+  </si>
+  <si>
+    <t>Items vacío, Unidades 0 y localStorage = '[]'</t>
+  </si>
+  <si>
+    <t>localStorage = '[]', Items vacío y Unidades 0</t>
+  </si>
+  <si>
+    <t>vaciarCarrito escribe '[]' en localStorage en lugar de eliminar la clave.</t>
+  </si>
+  <si>
+    <t>PU-004</t>
+  </si>
+  <si>
+    <t>CardProducto</t>
+  </si>
+  <si>
+    <t>agregarAlCarrito por click en 'Agregar al carro'</t>
+  </si>
+  <si>
+    <t>El producto se agrega al carrito al hacer click en 'Agregar al carro'</t>
+  </si>
+  <si>
+    <t>productoMock TC001; click en botón 'Agregar al carro'</t>
+  </si>
+  <si>
+    <t>localStorage['carrito'] contiene 1 item TC001</t>
+  </si>
+  <si>
+    <t>carrito vacío ([]): no se realizó el click antes de verificar</t>
+  </si>
+  <si>
+    <t>Falló</t>
+  </si>
+  <si>
+    <t>Paulo Riveros</t>
+  </si>
+  <si>
+    <t>El test verifica localStorage sin ejecutar fireEvent.click en 'Agregar al carro'; por eso el carrito queda []. Agregar el click antes del assert.</t>
+  </si>
+  <si>
+    <t>PU-005</t>
+  </si>
+  <si>
+    <t>Navegación - Link 'Ver producto'</t>
+  </si>
+  <si>
+    <t>El enlace 'Ver producto' navega a /producto/:codigo</t>
+  </si>
+  <si>
+    <t>productoMock TC001; click en 'Ver producto'</t>
+  </si>
+  <si>
+    <t>Se renderiza la página de detalle en /producto/TC001</t>
+  </si>
+  <si>
+    <t>Se muestra 'Página de Detalle del Producto'</t>
+  </si>
+  <si>
+    <t>PU-006</t>
+  </si>
+  <si>
+    <t>Autenticación</t>
+  </si>
+  <si>
+    <t>register(nuevoUsuario)</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>No permite registrar un usuario con un correo ya existente</t>
+  </si>
+  <si>
+    <t>usuario Ana con correo 'ana@correo.cl' ya registrado en localStorage</t>
+  </si>
+  <si>
+    <t>register retorna success:false con mensaje 'El correo ya se encuentra registrado'</t>
+  </si>
+  <si>
+    <t>Se muestra 'Resultado: El correo ya se encuentra registrado'</t>
+  </si>
   <si>
     <t>Registro de Pruebas Unitarias</t>
   </si>
@@ -132,162 +312,6 @@
     <t>• Caso de error: entrada inválida que debería lanzar excepción o devolver error.</t>
   </si>
   <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Módulo / Clase</t>
-  </si>
-  <si>
-    <t>Función / Método</t>
-  </si>
-  <si>
-    <t>Tipo de caso</t>
-  </si>
-  <si>
-    <t>Descripción del caso</t>
-  </si>
-  <si>
-    <t>Datos de entrada</t>
-  </si>
-  <si>
-    <t>Resultado esperado</t>
-  </si>
-  <si>
-    <t>Resultado obtenido</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Responsable</t>
-  </si>
-  <si>
-    <t>Fecha ejecución</t>
-  </si>
-  <si>
-    <t>Observaciones</t>
-  </si>
-  <si>
-    <t>PU-001</t>
-  </si>
-  <si>
-    <t>Carrito</t>
-  </si>
-  <si>
-    <t>agregarAlCarrito(codigo)</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>Agregar dos veces el mismo producto (TC001) deja una sola fila con cantidad 2</t>
-  </si>
-  <si>
-    <t>codigo: 'TC001' (dos clicks en 'Agregar Torta')</t>
-  </si>
-  <si>
-    <t>Una sola fila TC001 con cantidad 2 y totalUnidades = 2</t>
-  </si>
-  <si>
-    <t>Se muestra 'Items: TC001x2' y 'Unidades: 2'</t>
-  </si>
-  <si>
-    <t>Pasó</t>
-  </si>
-  <si>
-    <t>Joaquin Fuenzalida</t>
-  </si>
-  <si>
-    <t>PU-002</t>
-  </si>
-  <si>
-    <t>agregarAlCarrito - persistencia (localStorage)</t>
-  </si>
-  <si>
-    <t>El carrito se guarda en localStorage al agregar un producto</t>
-  </si>
-  <si>
-    <t>codigo: 'TC001'</t>
-  </si>
-  <si>
-    <t>localStorage['carrito'] contiene 1 item TC001 con cantidad 1</t>
-  </si>
-  <si>
-    <t>carrito = [{ codigo: 'TC001', cantidad: 1 }]</t>
-  </si>
-  <si>
-    <t>Paulo Riveros</t>
-  </si>
-  <si>
-    <t>PU-003</t>
-  </si>
-  <si>
-    <t>vaciarCarrito()</t>
-  </si>
-  <si>
-    <t>Borde</t>
-  </si>
-  <si>
-    <t>Vaciar el carrito deja el carrito y localStorage vacíos</t>
-  </si>
-  <si>
-    <t>Agregar TC001 y luego click en 'Vaciar'</t>
-  </si>
-  <si>
-    <t>Items vacío, Unidades 0 y localStorage = '[]'</t>
-  </si>
-  <si>
-    <t>localStorage = '[]', Items vacío y Unidades 0</t>
-  </si>
-  <si>
-    <t>vaciarCarrito escribe '[]' en localStorage en lugar de eliminar la clave.</t>
-  </si>
-  <si>
-    <t>PU-004</t>
-  </si>
-  <si>
-    <t>CardProducto</t>
-  </si>
-  <si>
-    <t>agregarAlCarrito por click en 'Agregar al carro'</t>
-  </si>
-  <si>
-    <t>El producto se agrega al carrito al hacer click en 'Agregar al carro'</t>
-  </si>
-  <si>
-    <t>productoMock TC001; click en botón 'Agregar al carro'</t>
-  </si>
-  <si>
-    <t>localStorage['carrito'] contiene 1 item TC001</t>
-  </si>
-  <si>
-    <t>carrito vacío ([]): no se realizó el click antes de verificar</t>
-  </si>
-  <si>
-    <t>Falló</t>
-  </si>
-  <si>
-    <t>El test verifica localStorage sin ejecutar fireEvent.click en 'Agregar al carro'; por eso el carrito queda []. Agregar el click antes del assert.</t>
-  </si>
-  <si>
-    <t>PU-005</t>
-  </si>
-  <si>
-    <t>Navegación - Link 'Ver producto'</t>
-  </si>
-  <si>
-    <t>El enlace 'Ver producto' navega a /producto/:codigo</t>
-  </si>
-  <si>
-    <t>productoMock TC001; click en 'Ver producto'</t>
-  </si>
-  <si>
-    <t>Se renderiza la página de detalle en /producto/TC001</t>
-  </si>
-  <si>
-    <t>Se muestra 'Página de Detalle del Producto'</t>
-  </si>
-  <si>
     <t>Resumen de Pruebas</t>
   </si>
   <si>
@@ -316,9 +340,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Error</t>
   </si>
   <si>
     <t>Esta hoja se calcula automáticamente desde 'Casos de Prueba'.</t>
@@ -344,40 +365,47 @@
       <sz val="16"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -765,86 +793,86 @@
     <col min="3" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>9</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -852,22 +880,22 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>18</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1875,238 +1903,260 @@
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="K2" s="10">
         <v>46304</v>
       </c>
       <c r="L2" s="8"/>
     </row>
-    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="K3" s="10">
         <v>46304</v>
       </c>
       <c r="L3" s="8"/>
     </row>
-    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="K4" s="10">
         <v>46304</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="K5" s="10">
         <v>46304</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="K6" s="10">
         <v>46304</v>
       </c>
       <c r="L6" s="8"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="10"/>
+    <row r="7" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="10">
+        <v>46304</v>
+      </c>
       <c r="L7" s="8"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -5664,32 +5714,32 @@
     <col min="5" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B3" s="11">
         <f>COUNTA('Casos de Prueba'!A2:A201)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="B5" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Falló")</f>
@@ -5698,7 +5748,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B6" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pendiente")</f>
@@ -5707,7 +5757,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Omitido")</f>
@@ -5716,7 +5766,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B8" s="11">
         <f>B3-SUM(B4:B7)</f>
@@ -5725,44 +5775,44 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B9" s="16">
         <f>IFERROR(B4/(B4+B5),0)</f>
-        <v>0.8</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B10" s="16">
         <f>IFERROR((B4+B5+B7)/B3,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="18" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="B15" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A15)</f>
@@ -5779,7 +5829,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="B16" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A16)</f>
@@ -5796,15 +5846,15 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="B17" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A17)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A17,'Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A17,'Casos de Prueba'!I2:I201,"Falló")</f>
@@ -5813,7 +5863,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
se añaden tests de login y categoria, se corrige test de cardProducto y se actualiza registro de pruebas
</commit_message>
<xml_diff>
--- a/Registro_Pruebas_Unitarias.xlsx
+++ b/Registro_Pruebas_Unitarias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moka/Documents/ReactPasteleria/ProyectoReactPasteleria/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738BECD4-3BAC-DA4F-9364-80FB319E7D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E46E009E-4D66-5B48-8D6A-BD4F4C73D322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="20000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="107">
   <si>
     <t>ID</t>
   </si>
@@ -183,7 +183,7 @@
     <t>agregarAlCarrito por click en 'Agregar al carro'</t>
   </si>
   <si>
-    <t>El producto se agrega al carrito al hacer click en 'Agregar al carro'</t>
+    <t>carrito = [{ codigo: 'TC001', cantidad: 1 }]: se ejecuta fireEvent.click en 'Agregar al carro'</t>
   </si>
   <si>
     <t>productoMock TC001; click en botón 'Agregar al carro'</t>
@@ -195,127 +195,169 @@
     <t>carrito vacío ([]): no se realizó el click antes de verificar</t>
   </si>
   <si>
+    <t>Paulo Riveros</t>
+  </si>
+  <si>
+    <t>Se agregó el fireEvent.click en 'Agregar al carro' antes del assert (cardProducto.test.jsx).</t>
+  </si>
+  <si>
+    <t>PU-005</t>
+  </si>
+  <si>
+    <t>Navegación - Link 'Ver producto'</t>
+  </si>
+  <si>
+    <t>El enlace 'Ver producto' navega a /producto/:codigo</t>
+  </si>
+  <si>
+    <t>productoMock TC001; click en 'Ver producto'</t>
+  </si>
+  <si>
+    <t>Se renderiza la página de detalle en /producto/TC001</t>
+  </si>
+  <si>
+    <t>Se muestra 'Página de Detalle del Producto'</t>
+  </si>
+  <si>
+    <t>PU-006</t>
+  </si>
+  <si>
+    <t>Autenticación</t>
+  </si>
+  <si>
+    <t>register(nuevoUsuario)</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>No permite registrar un usuario con un correo ya existente</t>
+  </si>
+  <si>
+    <t>usuario Ana con correo 'ana@correo.cl' ya registrado en localStorage</t>
+  </si>
+  <si>
+    <t>register retorna success:false con mensaje 'El correo ya se encuentra registrado'</t>
+  </si>
+  <si>
+    <t>Se muestra 'Resultado: El correo ya se encuentra registrado'</t>
+  </si>
+  <si>
+    <t>PU-007</t>
+  </si>
+  <si>
+    <t>ModalLogin</t>
+  </si>
+  <si>
+    <t>Validación de campos vacíos en handleSubmit</t>
+  </si>
+  <si>
+    <t>Enviar el formulario de login sin correo ni contraseña</t>
+  </si>
+  <si>
+    <t>Modal login abierto; click en 'Ingresar' sin llenar campos</t>
+  </si>
+  <si>
+    <t>Se muestra el mensaje 'debes ingresar tu correo y tu contraseña' y no se llama a login</t>
+  </si>
+  <si>
+    <t>Se muestra 'debes ingresar tu correo y tu contraseña'</t>
+  </si>
+  <si>
+    <t>PU-008</t>
+  </si>
+  <si>
+    <t>Catalogo</t>
+  </si>
+  <si>
+    <t>Filtrado por categoría (productosFiltrados)</t>
+  </si>
+  <si>
+    <t>Al seleccionar 'Productos Sin Azúcar' solo se muestran los productos de esa categoría</t>
+  </si>
+  <si>
+    <t>Click en 'Filtrar' con categoría 'Productos Sin Azúcar'</t>
+  </si>
+  <si>
+    <t>Título 'Productos Sin Azúcar' y 3 tarjetas (PSA001, PSA002, PSA003)</t>
+  </si>
+  <si>
+    <t>Título 'Productos Sin Azúcar' y 3 tarjetas de producto</t>
+  </si>
+  <si>
+    <t>Registro de Pruebas Unitarias</t>
+  </si>
+  <si>
+    <t>Proyecto:</t>
+  </si>
+  <si>
+    <t>Pasteleria Mil Sabores</t>
+  </si>
+  <si>
+    <t>Curso / Asignatura:</t>
+  </si>
+  <si>
+    <t>Desarrollo Fullstack II  Seccion 011D</t>
+  </si>
+  <si>
+    <t>Equipo / Integrantes:</t>
+  </si>
+  <si>
+    <t>Paulo Riveros - Marcelo Dervis - Joaquin Fuenzalida</t>
+  </si>
+  <si>
+    <t>Lenguaje y framework de pruebas:</t>
+  </si>
+  <si>
+    <t>HTML - JAVASCRIPT, REACT</t>
+  </si>
+  <si>
+    <t>Cómo usar esta planilla</t>
+  </si>
+  <si>
+    <t>1. Completen los datos del proyecto arriba (celdas amarillas).</t>
+  </si>
+  <si>
+    <t>2. En la hoja 'Casos de Prueba', agreguen una fila por cada caso de prueba (un test = una fila).</t>
+  </si>
+  <si>
+    <t>3. Las celdas amarillas son para completar; las filas 1–3 de ejemplo se pueden borrar o reemplazar.</t>
+  </si>
+  <si>
+    <t>4. Usen IDs correlativos: PU-001, PU-002, ... para poder referenciarlos en el informe.</t>
+  </si>
+  <si>
+    <t>5. 'Resultado esperado' se escribe ANTES de ejecutar; 'Resultado obtenido' DESPUÉS.</t>
+  </si>
+  <si>
+    <t>6. Elijan el Estado desde la lista: Pasó, Falló, Pendiente u Omitido.</t>
+  </si>
+  <si>
+    <t>7. Si un test falla, describan el error en 'Observaciones' y, al corregirlo, actualicen el estado.</t>
+  </si>
+  <si>
+    <t>8. La hoja 'Resumen' se calcula sola: no hay que escribir nada ahí.</t>
+  </si>
+  <si>
+    <t>Tipos de caso sugeridos:</t>
+  </si>
+  <si>
+    <t>• Caso normal: entrada válida típica.</t>
+  </si>
+  <si>
+    <t>• Caso borde: límites (0, vacío, máximo, mínimo, un solo elemento).</t>
+  </si>
+  <si>
+    <t>• Caso de error: entrada inválida que debería lanzar excepción o devolver error.</t>
+  </si>
+  <si>
+    <t>Resumen de Pruebas</t>
+  </si>
+  <si>
+    <t>Total de casos</t>
+  </si>
+  <si>
     <t>Falló</t>
-  </si>
-  <si>
-    <t>Paulo Riveros</t>
-  </si>
-  <si>
-    <t>El test verifica localStorage sin ejecutar fireEvent.click en 'Agregar al carro'; por eso el carrito queda []. Agregar el click antes del assert.</t>
-  </si>
-  <si>
-    <t>PU-005</t>
-  </si>
-  <si>
-    <t>Navegación - Link 'Ver producto'</t>
-  </si>
-  <si>
-    <t>El enlace 'Ver producto' navega a /producto/:codigo</t>
-  </si>
-  <si>
-    <t>productoMock TC001; click en 'Ver producto'</t>
-  </si>
-  <si>
-    <t>Se renderiza la página de detalle en /producto/TC001</t>
-  </si>
-  <si>
-    <t>Se muestra 'Página de Detalle del Producto'</t>
-  </si>
-  <si>
-    <t>PU-006</t>
-  </si>
-  <si>
-    <t>Autenticación</t>
-  </si>
-  <si>
-    <t>register(nuevoUsuario)</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>No permite registrar un usuario con un correo ya existente</t>
-  </si>
-  <si>
-    <t>usuario Ana con correo 'ana@correo.cl' ya registrado en localStorage</t>
-  </si>
-  <si>
-    <t>register retorna success:false con mensaje 'El correo ya se encuentra registrado'</t>
-  </si>
-  <si>
-    <t>Se muestra 'Resultado: El correo ya se encuentra registrado'</t>
-  </si>
-  <si>
-    <t>Registro de Pruebas Unitarias</t>
-  </si>
-  <si>
-    <t>Proyecto:</t>
-  </si>
-  <si>
-    <t>Pasteleria Mil Sabores</t>
-  </si>
-  <si>
-    <t>Curso / Asignatura:</t>
-  </si>
-  <si>
-    <t>Desarrollo Fullstack II  Seccion 011D</t>
-  </si>
-  <si>
-    <t>Equipo / Integrantes:</t>
-  </si>
-  <si>
-    <t>Paulo Riveros - Marcelo Dervis - Joaquin Fuenzalida</t>
-  </si>
-  <si>
-    <t>Lenguaje y framework de pruebas:</t>
-  </si>
-  <si>
-    <t>HTML - JAVASCRIPT, REACT</t>
-  </si>
-  <si>
-    <t>Cómo usar esta planilla</t>
-  </si>
-  <si>
-    <t>1. Completen los datos del proyecto arriba (celdas amarillas).</t>
-  </si>
-  <si>
-    <t>2. En la hoja 'Casos de Prueba', agreguen una fila por cada caso de prueba (un test = una fila).</t>
-  </si>
-  <si>
-    <t>3. Las celdas amarillas son para completar; las filas 1–3 de ejemplo se pueden borrar o reemplazar.</t>
-  </si>
-  <si>
-    <t>4. Usen IDs correlativos: PU-001, PU-002, ... para poder referenciarlos en el informe.</t>
-  </si>
-  <si>
-    <t>5. 'Resultado esperado' se escribe ANTES de ejecutar; 'Resultado obtenido' DESPUÉS.</t>
-  </si>
-  <si>
-    <t>6. Elijan el Estado desde la lista: Pasó, Falló, Pendiente u Omitido.</t>
-  </si>
-  <si>
-    <t>7. Si un test falla, describan el error en 'Observaciones' y, al corregirlo, actualicen el estado.</t>
-  </si>
-  <si>
-    <t>8. La hoja 'Resumen' se calcula sola: no hay que escribir nada ahí.</t>
-  </si>
-  <si>
-    <t>Tipos de caso sugeridos:</t>
-  </si>
-  <si>
-    <t>• Caso normal: entrada válida típica.</t>
-  </si>
-  <si>
-    <t>• Caso borde: límites (0, vacío, máximo, mínimo, un solo elemento).</t>
-  </si>
-  <si>
-    <t>• Caso de error: entrada inválida que debería lanzar excepción o devolver error.</t>
-  </si>
-  <si>
-    <t>Resumen de Pruebas</t>
-  </si>
-  <si>
-    <t>Total de casos</t>
   </si>
   <si>
     <t>Pendiente</t>
@@ -795,84 +837,84 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -880,22 +922,22 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2075,78 +2117,78 @@
         <v>42</v>
       </c>
       <c r="I5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>43</v>
-      </c>
-      <c r="J5" s="20" t="s">
-        <v>44</v>
       </c>
       <c r="K5" s="10">
         <v>46304</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K6" s="10">
         <v>46304</v>
       </c>
       <c r="L6" s="8"/>
     </row>
-    <row r="7" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>59</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>20</v>
@@ -2159,32 +2201,76 @@
       </c>
       <c r="L7" s="8"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="10"/>
+    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="10">
+        <v>46304</v>
+      </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="10"/>
+    <row r="9" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="10">
+        <v>46304</v>
+      </c>
       <c r="L9" s="8"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -5716,16 +5802,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="B3" s="11">
         <f>COUNTA('Casos de Prueba'!A2:A201)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -5734,21 +5820,21 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
       <c r="B5" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Falló")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="B6" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pendiente")</f>
@@ -5757,7 +5843,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Omitido")</f>
@@ -5766,7 +5852,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="B8" s="11">
         <f>B3-SUM(B4:B7)</f>
@@ -5775,16 +5861,16 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B9" s="16">
         <f>IFERROR(B4/(B4+B5),0)</f>
-        <v>0.83333333333333337</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B10" s="16">
         <f>IFERROR((B4+B5+B7)/B3,0)</f>
@@ -5793,21 +5879,21 @@
     </row>
     <row r="13" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -5816,15 +5902,15 @@
       </c>
       <c r="B15" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A15)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Falló")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -5833,11 +5919,11 @@
       </c>
       <c r="B16" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A16)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A16,'Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A16,'Casos de Prueba'!I2:I201,"Falló")</f>
@@ -5846,7 +5932,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A17)</f>
@@ -5863,7 +5949,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Agrega test de eliminar producto y recuperar contraseña, registra casos PU-009 y PU-010 en la planilla
</commit_message>
<xml_diff>
--- a/Registro_Pruebas_Unitarias.xlsx
+++ b/Registro_Pruebas_Unitarias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moka/Documents/ReactPasteleria/ProyectoReactPasteleria/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E46E009E-4D66-5B48-8D6A-BD4F4C73D322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E30E3C3-310A-DF4D-8429-7D2DC17D8882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="20000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="119">
   <si>
     <t>ID</t>
   </si>
@@ -283,6 +283,42 @@
   </si>
   <si>
     <t>Título 'Productos Sin Azúcar' y 3 tarjetas de producto</t>
+  </si>
+  <si>
+    <t>PU-009</t>
+  </si>
+  <si>
+    <t>eliminarDelCarrito(codigo)</t>
+  </si>
+  <si>
+    <t>Eliminar un producto lo quita del carrito (UI y localStorage)</t>
+  </si>
+  <si>
+    <t>Agregar TC001 y luego click en 'Eliminar producto'</t>
+  </si>
+  <si>
+    <t>Se muestra 'Items: vacío' y localStorage['carrito'] = []</t>
+  </si>
+  <si>
+    <t>localStorage = [] y se muestra 'Items: vacío'</t>
+  </si>
+  <si>
+    <t>PU-010</t>
+  </si>
+  <si>
+    <t>recuperarPassword(correo)</t>
+  </si>
+  <si>
+    <t>recuperarPassword devuelve la contraseña de un correo registrado</t>
+  </si>
+  <si>
+    <t>Usuario en localStorage con correo 'ana@correo.cl' y password 'Doki21431.@'</t>
+  </si>
+  <si>
+    <t>Se muestra 'Resultado: Doki21431.@'</t>
+  </si>
+  <si>
+    <t>Se muestra la contraseña del usuario registrado</t>
   </si>
   <si>
     <t>Registro de Pruebas Unitarias</t>
@@ -837,84 +873,84 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -922,22 +958,22 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2201,7 +2237,7 @@
       </c>
       <c r="L7" s="8"/>
     </row>
-    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -2237,7 +2273,7 @@
       </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>66</v>
       </c>
@@ -2273,32 +2309,76 @@
       </c>
       <c r="L9" s="8"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="10"/>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="10">
+        <v>46306</v>
+      </c>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="10"/>
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A11" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="10">
+        <v>46306</v>
+      </c>
       <c r="L11" s="8"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -5802,16 +5882,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="B3" s="11">
         <f>COUNTA('Casos de Prueba'!A2:A201)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -5820,12 +5900,12 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="B5" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Falló")</f>
@@ -5834,7 +5914,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B6" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Pendiente")</f>
@@ -5843,7 +5923,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Casos de Prueba'!I2:I201,"Omitido")</f>
@@ -5852,7 +5932,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B8" s="11">
         <f>B3-SUM(B4:B7)</f>
@@ -5861,7 +5941,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B9" s="16">
         <f>IFERROR(B4/(B4+B5),0)</f>
@@ -5870,7 +5950,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B10" s="16">
         <f>IFERROR((B4+B5+B7)/B3,0)</f>
@@ -5879,21 +5959,21 @@
     </row>
     <row r="13" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -5902,11 +5982,11 @@
       </c>
       <c r="B15" s="11">
         <f>COUNTIF('Casos de Prueba'!D2:D201,A15)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C15" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Pasó")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" s="11">
         <f>COUNTIFS('Casos de Prueba'!D2:D201,A15,'Casos de Prueba'!I2:I201,"Falló")</f>
@@ -5949,7 +6029,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>